<commit_message>
Atualizando data/season_2026/next_games/next_games.xlsx via script
</commit_message>
<xml_diff>
--- a/data/season_2026/next_games/next_games.xlsx
+++ b/data/season_2026/next_games/next_games.xlsx
@@ -573,27 +573,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>10.72</t>
+          <t>11.02</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>6.59</t>
+          <t>6.64</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t>1.22</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>1.53</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2.37</t>
         </is>
       </c>
       <c r="N2" t="inlineStr"/>
@@ -628,7 +628,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2.30</t>
+          <t>2.45</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -640,22 +640,22 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>3.30</t>
+          <t>3.10</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2.37</t>
+          <t>2.52</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>3.07</t>
+          <t>3.13</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>3.56</t>
+          <t>3.18</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -881,17 +881,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>9.52</t>
+          <t>9.83</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>6.05</t>
+          <t>6.16</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t>1.24</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1021,17 +1021,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>1.86</t>
+          <t>1.88</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>3.43</t>
+          <t>3.47</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>4.21</t>
+          <t>4.26</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1058,13 +1058,13 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1.92</t>
+          <t>1.93</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1.86</t>
+          <t>1.87</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
@@ -1088,7 +1088,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3.70</t>
+          <t>3.50</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -1100,12 +1100,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2.35</t>
+          <t>2.45</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>3.48</t>
+          <t>3.38</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2.35</t>
+          <t>2.46</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>1.48</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -1168,12 +1168,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>4.75</t>
+          <t>5.00</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>1.49</t>
+          <t>1.51</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>4.92</t>
+          <t>4.99</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1197,13 +1197,29 @@
         </is>
       </c>
       <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
       <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1.80</t>
+        </is>
+      </c>
       <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
       <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>1.82</t>
+        </is>
+      </c>
       <c r="V10" t="inlineStr"/>
     </row>
     <row r="11">
@@ -1297,17 +1313,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>8.14</t>
+          <t>8.39</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>4.41</t>
+          <t>4.51</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>1.41</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1375,7 +1391,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>4.47</t>
+          <t>4.48</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1433,17 +1449,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1.86</t>
+          <t>1.88</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>3.65</t>
+          <t>3.69</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>4.12</t>
+          <t>4.17</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1470,13 +1486,13 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>2.05</t>
+          <t>2.06</t>
         </is>
       </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.82</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
@@ -1522,12 +1538,12 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>7.89</t>
+          <t>7.84</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>16.14</t>
+          <t>15.91</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1585,17 +1601,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2.10</t>
+          <t>2.08</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>3.57</t>
+          <t>3.58</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>3.59</t>
+          <t>3.64</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1669,17 +1685,17 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>3.15</t>
+          <t>3.08</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>3.62</t>
+          <t>3.58</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2.19</t>
+          <t>2.24</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1753,17 +1769,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2.36</t>
+          <t>2.37</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>3.04</t>
+          <t>3.08</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>3.24</t>
+          <t>3.27</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1821,17 +1837,17 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.95</t>
+          <t>1.93</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>3.42</t>
+          <t>3.43</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>3.88</t>
+          <t>3.91</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -2030,12 +2046,12 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2.80</t>
+          <t>2.81</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2.52</t>
+          <t>2.51</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -2161,17 +2177,17 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>1.45</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>4.85</t>
+          <t>4.90</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>6.19</t>
+          <t>6.26</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -2229,17 +2245,17 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>3.28</t>
+          <t>3.29</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>3.86</t>
+          <t>3.81</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2.05</t>
+          <t>2.07</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -3569,7 +3585,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2.80</t>
+          <t>2.78</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -3579,7 +3595,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2.70</t>
+          <t>2.72</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -4268,7 +4284,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>2.15</t>
+          <t>2.20</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -4280,12 +4296,12 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>2.80</t>
+          <t>2.70</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2.26</t>
+          <t>2.35</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -4295,7 +4311,7 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>2.88</t>
+          <t>2.74</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -4734,22 +4750,22 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>7.02</t>
+          <t>7.15</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>13.20</t>
+          <t>13.66</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>1.53</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2.37</t>
         </is>
       </c>
       <c r="N60" t="inlineStr"/>
@@ -5921,17 +5937,17 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2.61</t>
+          <t>2.62</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>2.97</t>
+          <t>2.98</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>3.19</t>
+          <t>3.17</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
@@ -5972,7 +5988,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>4.75</t>
+          <t>4.50</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
@@ -5984,22 +6000,22 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1.83</t>
+          <t>1.90</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>5.20</t>
+          <t>5.14</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>3.32</t>
+          <t>3.30</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>1.85</t>
+          <t>1.86</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
@@ -6108,7 +6124,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>2.87</t>
+          <t>2.80</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -6120,12 +6136,12 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>2.40</t>
+          <t>2.45</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2.91</t>
+          <t>2.92</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -6140,12 +6156,12 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>2.20</t>
+          <t>2.10</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>1.61</t>
+          <t>1.66</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -6234,13 +6250,13 @@
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>1.85</t>
+          <t>1.82</t>
         </is>
       </c>
       <c r="O81" t="inlineStr"/>
       <c r="P81" t="inlineStr">
         <is>
-          <t>2.00</t>
+          <t>2.02</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr"/>
@@ -6293,7 +6309,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2.64</t>
+          <t>2.59</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -6303,7 +6319,7 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>2.77</t>
+          <t>2.83</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
@@ -6817,17 +6833,17 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>7.43</t>
+          <t>7.75</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>4.65</t>
+          <t>4.75</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>1.45</t>
+          <t>1.43</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
@@ -7089,17 +7105,17 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2.13</t>
+          <t>2.12</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>3.21</t>
+          <t>3.25</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>3.74</t>
+          <t>3.72</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
@@ -7126,13 +7142,13 @@
       <c r="Q93" t="inlineStr"/>
       <c r="R93" t="inlineStr">
         <is>
-          <t>2.00</t>
+          <t>1.95</t>
         </is>
       </c>
       <c r="S93" t="inlineStr"/>
       <c r="T93" t="inlineStr">
         <is>
-          <t>1.84</t>
+          <t>1.88</t>
         </is>
       </c>
       <c r="U93" t="inlineStr"/>
@@ -7455,7 +7471,7 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>6.28</t>
+          <t>6.27</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -7539,7 +7555,7 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>4.15</t>
+          <t>4.16</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -7567,7 +7583,7 @@
       <c r="R99" t="inlineStr"/>
       <c r="S99" t="inlineStr">
         <is>
-          <t>1.95</t>
+          <t>1.96</t>
         </is>
       </c>
       <c r="T99" t="inlineStr"/>
@@ -7613,12 +7629,12 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>2.19</t>
+          <t>2.20</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>3.67</t>
+          <t>3.66</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -7765,12 +7781,12 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>1.90</t>
+          <t>1.89</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>4.29</t>
+          <t>4.31</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -7849,17 +7865,17 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>1.88</t>
+          <t>1.86</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
+          <t>3.89</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
           <t>3.86</t>
-        </is>
-      </c>
-      <c r="K103" t="inlineStr">
-        <is>
-          <t>3.84</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -8069,17 +8085,17 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>2.06</t>
+          <t>2.10</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>2.91</t>
+          <t>2.87</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>4.48</t>
+          <t>4.43</t>
         </is>
       </c>
       <c r="L106" t="inlineStr">
@@ -8278,12 +8294,12 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>3.49</t>
+          <t>3.50</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>3.34</t>
+          <t>3.33</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -8310,13 +8326,13 @@
       <c r="Q109" t="inlineStr"/>
       <c r="R109" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.82</t>
         </is>
       </c>
       <c r="S109" t="inlineStr"/>
       <c r="T109" t="inlineStr">
         <is>
-          <t>2.03</t>
+          <t>2.02</t>
         </is>
       </c>
       <c r="U109" t="inlineStr"/>
@@ -8509,17 +8525,17 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>1.47</t>
+          <t>1.46</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>4.87</t>
+          <t>4.89</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>5.93</t>
+          <t>5.99</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
@@ -8661,17 +8677,17 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>2.01</t>
+          <t>2.00</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>3.78</t>
+          <t>3.80</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>3.46</t>
+          <t>3.48</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
@@ -9377,17 +9393,17 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>1.76</t>
+          <t>1.80</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>4.17</t>
+          <t>4.11</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>4.09</t>
+          <t>3.94</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
@@ -9666,7 +9682,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>5.04</t>
+          <t>5.02</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -10290,22 +10306,22 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>3.79</t>
+          <t>3.78</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>4.21</t>
+          <t>4.18</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>1.95</t>
+          <t>2.00</t>
         </is>
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>1.80</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="N138" t="inlineStr">
@@ -10841,12 +10857,12 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>7.58</t>
+          <t>7.56</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>4.73</t>
+          <t>4.72</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -11345,7 +11361,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>2.17</t>
+          <t>2.18</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
@@ -11355,7 +11371,7 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>4.15</t>
+          <t>4.12</t>
         </is>
       </c>
       <c r="L153" t="inlineStr">
@@ -11481,17 +11497,17 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>2.59</t>
+          <t>2.70</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>2.86</t>
+          <t>2.84</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>3.18</t>
+          <t>3.07</t>
         </is>
       </c>
       <c r="L155" t="inlineStr">
@@ -12099,7 +12115,7 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>5.93</t>
+          <t>5.94</t>
         </is>
       </c>
       <c r="L163" t="inlineStr">
@@ -12241,17 +12257,17 @@
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>2.52</t>
+          <t>2.53</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>3.24</t>
+          <t>3.21</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>2.92</t>
+          <t>2.93</t>
         </is>
       </c>
       <c r="L165" t="inlineStr">
@@ -12278,13 +12294,13 @@
       <c r="Q165" t="inlineStr"/>
       <c r="R165" t="inlineStr">
         <is>
-          <t>1.99</t>
+          <t>2.03</t>
         </is>
       </c>
       <c r="S165" t="inlineStr"/>
       <c r="T165" t="inlineStr">
         <is>
-          <t>1.84</t>
+          <t>1.81</t>
         </is>
       </c>
       <c r="U165" t="inlineStr"/>
@@ -12325,12 +12341,12 @@
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.74</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>3.84</t>
+          <t>3.80</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -12350,13 +12366,13 @@
       </c>
       <c r="N166" t="inlineStr">
         <is>
-          <t>1.87</t>
+          <t>1.92</t>
         </is>
       </c>
       <c r="O166" t="inlineStr"/>
       <c r="P166" t="inlineStr">
         <is>
-          <t>1.97</t>
+          <t>1.92</t>
         </is>
       </c>
       <c r="Q166" t="inlineStr"/>
@@ -12749,17 +12765,17 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>1.82</t>
+          <t>1.78</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>3.33</t>
+          <t>3.36</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>4.90</t>
+          <t>5.13</t>
         </is>
       </c>
       <c r="L172" t="inlineStr">
@@ -12817,17 +12833,17 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>2.33</t>
+          <t>2.28</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>3.74</t>
+          <t>3.80</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>2.82</t>
+          <t>2.87</t>
         </is>
       </c>
       <c r="L173" t="inlineStr">
@@ -12958,12 +12974,12 @@
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>3.36</t>
+          <t>3.33</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>2.06</t>
+          <t>2.07</t>
         </is>
       </c>
       <c r="L175" t="inlineStr">
@@ -13181,17 +13197,17 @@
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>1.65</t>
+          <t>1.62</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>3.53</t>
+          <t>3.60</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>6.01</t>
+          <t>6.13</t>
         </is>
       </c>
       <c r="L178" t="inlineStr">
@@ -13254,22 +13270,22 @@
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>2.98</t>
+          <t>2.99</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>2.51</t>
+          <t>2.50</t>
         </is>
       </c>
       <c r="L179" t="inlineStr">
         <is>
-          <t>1.66</t>
+          <t>1.70</t>
         </is>
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>2.10</t>
+          <t>2.05</t>
         </is>
       </c>
       <c r="N179" t="inlineStr"/>
@@ -14002,13 +14018,13 @@
       </c>
       <c r="N190" t="inlineStr">
         <is>
-          <t>1.90</t>
+          <t>1.87</t>
         </is>
       </c>
       <c r="O190" t="inlineStr"/>
       <c r="P190" t="inlineStr">
         <is>
-          <t>1.90</t>
+          <t>1.92</t>
         </is>
       </c>
       <c r="Q190" t="inlineStr"/>
@@ -14304,12 +14320,12 @@
       </c>
       <c r="L195" t="inlineStr">
         <is>
-          <t>1.90</t>
+          <t>1.80</t>
         </is>
       </c>
       <c r="M195" t="inlineStr">
         <is>
-          <t>1.90</t>
+          <t>1.95</t>
         </is>
       </c>
       <c r="N195" t="inlineStr">
@@ -14373,7 +14389,7 @@
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>3.79</t>
+          <t>3.81</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
@@ -14524,12 +14540,12 @@
       </c>
       <c r="L198" t="inlineStr">
         <is>
-          <t>1.61</t>
+          <t>1.66</t>
         </is>
       </c>
       <c r="M198" t="inlineStr">
         <is>
-          <t>2.20</t>
+          <t>2.10</t>
         </is>
       </c>
       <c r="N198" t="inlineStr"/>
@@ -14789,17 +14805,17 @@
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>2.32</t>
+          <t>2.31</t>
         </is>
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>3.00</t>
+          <t>3.03</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>3.53</t>
+          <t>3.52</t>
         </is>
       </c>
       <c r="L202" t="inlineStr">
@@ -14816,9 +14832,17 @@
       <c r="O202" t="inlineStr"/>
       <c r="P202" t="inlineStr"/>
       <c r="Q202" t="inlineStr"/>
-      <c r="R202" t="inlineStr"/>
+      <c r="R202" t="inlineStr">
+        <is>
+          <t>2.03</t>
+        </is>
+      </c>
       <c r="S202" t="inlineStr"/>
-      <c r="T202" t="inlineStr"/>
+      <c r="T202" t="inlineStr">
+        <is>
+          <t>1.81</t>
+        </is>
+      </c>
       <c r="U202" t="inlineStr"/>
       <c r="V202" t="inlineStr"/>
     </row>

</xml_diff>